<commit_message>
Add .gitignore and update project dependencies
</commit_message>
<xml_diff>
--- a/Mass_Balance_Calculator_Pro.xlsx
+++ b/Mass_Balance_Calculator_Pro.xlsx
@@ -62,10 +62,10 @@
   </si>
   <si>
     <t>INSTRUCTIONS:
-1. Enter experimental data in YELLOW cells.
-2. Default values provided for testing.
-3. Navigate to 'Diagnostic Report' tab to see analysis.
-4. Use 'Trend Tracking' for stability studies.</t>
+1. Enter your experimental data in the YELLOW cells.
+2. I've put in some default values just for testing.
+3. Once you're done, check the 'Diagnostic Report' tab for the analysis.
+4. 'Trend Tracking' is there if you're doing a stability study.</t>
   </si>
   <si>
     <t>GO TO REPORT &gt;&gt;</t>

</xml_diff>